<commit_message>
Draft Europe and Asia-Pacific region pages; metadata, hreflang rows, decision sheet row, tracker Z102-Z105, D93-D94; package refreshed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VNwEiodB4b8PQoyyzgGhFp
</commit_message>
<xml_diff>
--- a/outreach/editor-decision-sheet.xlsx
+++ b/outreach/editor-decision-sheet.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Decisions" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$4:$J$36</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$4:$J$37</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="153">
   <si>
     <t xml:space="preserve">Editor decision sheet: hotel records (Solo5Estrellas)</t>
   </si>
@@ -467,6 +467,21 @@
   </si>
   <si>
     <t xml:space="preserve">Generate every count from the list at render time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/regions/8/ and /regions/4/ (also chain pages)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Westin Miyako Kyoto (recorded in China); Andaz Singapore (China); Grand Hyatt Singapore (Malaysia); The Majestic Hotel Kuala Lumpur (India); Aleenta Resort &amp; Spa Phuket (Malaysia); Yiu Teung Mansion, Chengdu (Saint Lucia); Le Louise Brussels - MGallery (Germany)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country in the hotel record does not match the city</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correct the country at the record</t>
   </si>
 </sst>
 </file>
@@ -589,11 +604,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -906,32 +921,32 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -963,7 +978,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -991,7 +1006,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -1019,7 +1034,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -1047,7 +1062,7 @@
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
@@ -1075,7 +1090,7 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -1103,7 +1118,7 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
@@ -1131,7 +1146,7 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
@@ -1159,7 +1174,7 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
@@ -1187,7 +1202,7 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -1215,7 +1230,7 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
@@ -1243,7 +1258,7 @@
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
@@ -1271,7 +1286,7 @@
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
@@ -1299,7 +1314,7 @@
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
@@ -1327,7 +1342,7 @@
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
@@ -1355,7 +1370,7 @@
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
     </row>
-    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
@@ -1383,7 +1398,7 @@
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
     </row>
-    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
@@ -1411,7 +1426,7 @@
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
@@ -1439,7 +1454,7 @@
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
     </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
@@ -1467,7 +1482,7 @@
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
@@ -1495,7 +1510,7 @@
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
     </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
@@ -1523,7 +1538,7 @@
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
     </row>
-    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
         <v>21</v>
       </c>
@@ -1551,7 +1566,7 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
     </row>
-    <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
         <v>22</v>
       </c>
@@ -1579,7 +1594,7 @@
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
@@ -1607,7 +1622,7 @@
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
         <v>24</v>
       </c>
@@ -1635,7 +1650,7 @@
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
     </row>
-    <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
         <v>25</v>
       </c>
@@ -1663,7 +1678,7 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
         <v>26</v>
       </c>
@@ -1691,7 +1706,7 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
@@ -1719,7 +1734,7 @@
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
         <v>28</v>
       </c>
@@ -1747,7 +1762,7 @@
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
     </row>
-    <row r="33" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="n">
         <v>29</v>
       </c>
@@ -1775,7 +1790,7 @@
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
         <v>30</v>
       </c>
@@ -1803,7 +1818,7 @@
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
         <v>31</v>
       </c>
@@ -1831,7 +1846,7 @@
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
     </row>
-    <row r="36" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
         <v>32</v>
       </c>
@@ -1859,10 +1874,38 @@
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
     </row>
+    <row r="37" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J36"/>
+  <autoFilter ref="A4:J37"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I37" type="list">
       <formula1>"Remove,Keep one,Keep as is,Keep,Hold,Fix,Reassign brand,Confirm,Need more info"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Draft ten more region pages (Africa, Oceania, El Caribe, Centroamerica, Norteamerica, Sudamerica, Hawai, Mexico, Canada, Oriente Medio); region builder; metadata, hreflang, decision sheet, tracker Z106-Z109, D95-D104; package refreshed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VNwEiodB4b8PQoyyzgGhFp
</commit_message>
<xml_diff>
--- a/outreach/editor-decision-sheet.xlsx
+++ b/outreach/editor-decision-sheet.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Decisions" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$4:$J$37</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$4:$J$39</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="164">
   <si>
     <t xml:space="preserve">Editor decision sheet: hotel records (Solo5Estrellas)</t>
   </si>
@@ -482,6 +482,39 @@
   </si>
   <si>
     <t xml:space="preserve">Correct the country at the record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z109</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/regions/15/ Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thompson Zihuatanejo (recorded in Mongolia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correct the country to Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrong region page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/regions/10/, /regions/3/, /regions/18/, /regions/13/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Norteamérica lists 8 Canadian, 8 Mexican, 1 Puerto Rican and 1 French hotel (La Caserne Chanzy, Reims); Africa lists 4 hotels in Jordan; Oriente Medio lists 3 in Azerbaijan and 6 in India; Sudamérica lists Alexander Hotel (Mexico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotels sit on a region page that does not match their country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reassign region / Keep as is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assign each hotel to the region of its country; decide the region of Azerbaijan, Georgia, Kazakhstan, Turkey and Russia</t>
   </si>
 </sst>
 </file>
@@ -921,7 +954,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -1874,7 +1907,7 @@
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
     </row>
-    <row r="37" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
         <v>33</v>
       </c>
@@ -1902,11 +1935,67 @@
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
     </row>
+    <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+    </row>
+    <row r="39" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J37"/>
+  <autoFilter ref="A4:J39"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I37" type="list">
-      <formula1>"Remove,Keep one,Keep as is,Keep,Hold,Fix,Reassign brand,Confirm,Need more info"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I39" type="list">
+      <formula1>"Remove,Keep one,Keep as is,Keep,Hold,Fix,Reassign brand,Reassign region,Confirm,Need more info"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Draft 131 country pages; region pages refreshed (city names, single-country layout); hreflang map 213 rows; decision sheet 37 rows; tracker Z111-Z113, D106; package refreshed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VNwEiodB4b8PQoyyzgGhFp
</commit_message>
<xml_diff>
--- a/outreach/editor-decision-sheet.xlsx
+++ b/outreach/editor-decision-sheet.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Decisions" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$4:$J$39</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Decisions!$A$4:$J$41</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="178">
   <si>
     <t xml:space="preserve">Editor decision sheet: hotel records (Solo5Estrellas)</t>
   </si>
@@ -515,6 +515,48 @@
   </si>
   <si>
     <t xml:space="preserve">Assign each hotel to the region of its country; decide the region of Azerbaijan, Georgia, Kazakhstan, Turkey and Russia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duplicate or empty country records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/countries/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kuwait (IDs 141, 145, 147); Bhutan (74 'Buthan', 82 'Kingdom of Bhutan'); Serbia (143, 148); Mongolia (154, 155); Scotland (71) vs United Kingdom (157); 19 country IDs with no hotels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The same country exists under several IDs; empty countries still serve a page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merge / Keep as is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merge each duplicate into one ID (141, 82, 148, 154); decide whether Scotland stays separate; 404 the empty ones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country and region overlap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z113</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/countries/40/, /15/, /67/ and /regions/14/, /15/, /16/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">México, Canadá and Hawái exist as both a country (or part of one) and a region page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two pages list the same hotels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick canonical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep the country pages as canonical and point the region pages to them</t>
   </si>
 </sst>
 </file>
@@ -954,7 +996,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -1935,7 +1977,7 @@
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
     </row>
-    <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="n">
         <v>35</v>
       </c>
@@ -1963,7 +2005,7 @@
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
     </row>
-    <row r="39" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
         <v>36</v>
       </c>
@@ -1991,11 +2033,67 @@
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
     </row>
+    <row r="40" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+    </row>
+    <row r="41" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J39"/>
+  <autoFilter ref="A4:J41"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I39" type="list">
-      <formula1>"Remove,Keep one,Keep as is,Keep,Hold,Fix,Reassign brand,Reassign region,Confirm,Need more info"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I41" type="list">
+      <formula1>"Remove,Keep one,Keep as is,Keep,Hold,Fix,Reassign brand,Reassign region,Merge,Pick canonical,Confirm,Need more info"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>